<commit_message>
Decision makers: a people file with the people columns, contactless people to review, honest completion sentence, stricter industry evidence, richer lookup identity
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01ThHHQr9Z1VyJt99webNbFx
</commit_message>
<xml_diff>
--- a/public/samples/diger-sample-decision-makers.xlsx
+++ b/public/samples/diger-sample-decision-makers.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="45">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="42">
   <si>
     <t>نموذج توضيحي ببيانات وهمية</t>
   </si>
@@ -34,30 +34,27 @@
     <t>الشركة</t>
   </si>
   <si>
+    <t>الدولة</t>
+  </si>
+  <si>
+    <t>البريد المهني</t>
+  </si>
+  <si>
+    <t>حالة تحقق البريد المهني</t>
+  </si>
+  <si>
+    <t>رقم الهاتف</t>
+  </si>
+  <si>
+    <t>حالة تحقق الهاتف</t>
+  </si>
+  <si>
+    <t>لينكد إن</t>
+  </si>
+  <si>
     <t>مجال النشاط</t>
   </si>
   <si>
-    <t>الدولة / الموقع</t>
-  </si>
-  <si>
-    <t>لينكد إن</t>
-  </si>
-  <si>
-    <t>البريد المهني</t>
-  </si>
-  <si>
-    <t>رقم الهاتف</t>
-  </si>
-  <si>
-    <t>حالة الحقول</t>
-  </si>
-  <si>
-    <t>حالة تحقق البريد المهني</t>
-  </si>
-  <si>
-    <t>حالة تحقق الهاتف</t>
-  </si>
-  <si>
     <t>اسم تجريبي أ</t>
   </si>
   <si>
@@ -67,25 +64,19 @@
     <t>شركة النموذج الأولى</t>
   </si>
   <si>
+    <t>مصر</t>
+  </si>
+  <si>
+    <t>غير متاح</t>
+  </si>
+  <si>
+    <t>+201000000000</t>
+  </si>
+  <si>
+    <t>لم يتوفر تأكيد</t>
+  </si>
+  <si>
     <t>مقاولات</t>
-  </si>
-  <si>
-    <t>مصر</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
-    <t>غير متاح</t>
-  </si>
-  <si>
-    <t>+201000000000</t>
-  </si>
-  <si>
-    <t>البريد: غير موجود • الهاتف: موجود</t>
-  </si>
-  <si>
-    <t>لم يتوفر تأكيد</t>
   </si>
   <si>
     <t>اسم تجريبي ب</t>
@@ -601,21 +592,22 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:K10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="27" customWidth="1"/>
-    <col min="4" max="4" width="28" customWidth="1"/>
-    <col min="5" max="6" width="24" customWidth="1"/>
-    <col min="7" max="8" width="34" customWidth="1"/>
-    <col min="9" max="9" width="22" customWidth="1"/>
-    <col min="10" max="10" width="32" customWidth="1"/>
-    <col min="11" max="12" width="30" customWidth="1"/>
+    <col min="4" max="4" width="30" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="34" customWidth="1"/>
+    <col min="7" max="8" width="22" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+    <col min="10" max="10" width="34" customWidth="1"/>
+    <col min="11" max="11" width="28" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" ht="36" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" ht="36" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -629,9 +621,8 @@
       <c r="I1" s="1"/>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
-      <c r="L1" s="1"/>
     </row>
-    <row r="2" ht="28" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="2" ht="28" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -645,7 +636,6 @@
       <c r="I2" s="2"/>
       <c r="J2" s="2"/>
       <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
     </row>
     <row r="3" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
@@ -655,7 +645,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="4" ht="30" customHeight="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="4" ht="30" customHeight="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A4" s="3" t="s">
         <v>3</v>
       </c>
@@ -689,243 +679,222 @@
       <c r="K4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="L4" s="3" t="s">
-        <v>14</v>
-      </c>
     </row>
-    <row r="5" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="5" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A5" s="5">
         <v>1</v>
       </c>
       <c r="B5" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C5" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="D5" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>18</v>
-      </c>
       <c r="F5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G5" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H5" s="6" t="s">
         <v>19</v>
       </c>
-      <c r="G5" s="5" t="s">
+      <c r="I5" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H5" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="6" t="s">
-        <v>22</v>
-      </c>
       <c r="J5" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="L5" s="5" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="6" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="6" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A6" s="7">
         <v>2</v>
       </c>
       <c r="B6" s="7" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" s="7" t="s">
+        <v>23</v>
+      </c>
+      <c r="D6" s="7" t="s">
+        <v>24</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G6" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H6" s="8" t="s">
         <v>25</v>
       </c>
-      <c r="C6" s="7" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="7" t="s">
-        <v>27</v>
-      </c>
-      <c r="E6" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F6" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G6" s="7" t="s">
+      <c r="I6" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H6" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I6" s="8" t="s">
-        <v>28</v>
-      </c>
       <c r="J6" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L6" s="7" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="7" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="7" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A7" s="5">
         <v>3</v>
       </c>
       <c r="B7" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>28</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G7" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H7" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="C7" s="5" t="s">
-        <v>30</v>
-      </c>
-      <c r="D7" s="5" t="s">
-        <v>31</v>
-      </c>
-      <c r="E7" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F7" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G7" s="5" t="s">
+      <c r="I7" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H7" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I7" s="6" t="s">
-        <v>32</v>
-      </c>
       <c r="J7" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="L7" s="5" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="8" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="8" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A8" s="7">
         <v>4</v>
       </c>
       <c r="B8" s="7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>31</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H8" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="C8" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="D8" s="7" t="s">
-        <v>35</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G8" s="7" t="s">
+      <c r="I8" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H8" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I8" s="8" t="s">
-        <v>36</v>
-      </c>
       <c r="J8" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L8" s="7" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="9" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="9" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A9" s="5">
         <v>5</v>
       </c>
       <c r="B9" s="5" t="s">
+        <v>34</v>
+      </c>
+      <c r="C9" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="D9" s="5" t="s">
+        <v>36</v>
+      </c>
+      <c r="E9" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="F9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="G9" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="H9" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="C9" s="5" t="s">
-        <v>38</v>
-      </c>
-      <c r="D9" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>18</v>
-      </c>
-      <c r="F9" s="5" t="s">
-        <v>19</v>
-      </c>
-      <c r="G9" s="5" t="s">
+      <c r="I9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="5" t="s">
-        <v>21</v>
-      </c>
-      <c r="I9" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="J9" s="5" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K9" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="L9" s="5" t="s">
-        <v>24</v>
-      </c>
     </row>
-    <row r="10" ht="24" customHeight="1" spans="1:12" s="4" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="10" ht="24" customHeight="1" spans="1:11" s="4" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A10" s="7">
         <v>6</v>
       </c>
       <c r="B10" s="7" t="s">
+        <v>38</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>39</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>40</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="G10" s="7" t="s">
+        <v>18</v>
+      </c>
+      <c r="H10" s="8" t="s">
         <v>41</v>
       </c>
-      <c r="C10" s="7" t="s">
-        <v>42</v>
-      </c>
-      <c r="D10" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="E10" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="F10" s="7" t="s">
-        <v>19</v>
-      </c>
-      <c r="G10" s="7" t="s">
+      <c r="I10" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="H10" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I10" s="8" t="s">
-        <v>44</v>
-      </c>
       <c r="J10" s="7" t="s">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="L10" s="7" t="s">
-        <v>24</v>
-      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A4:L10"/>
+  <autoFilter ref="A4:K10"/>
   <mergeCells count="2">
-    <mergeCell ref="A1:L1"/>
-    <mergeCell ref="A2:L2"/>
+    <mergeCell ref="A1:K1"/>
+    <mergeCell ref="A2:K2"/>
   </mergeCells>
   <pageSetup paperSize="9" orientation="landscape" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="0" firstPageNumber="1" useFirstPageNumber="1" copies="1"/>
 </worksheet>

</xml_diff>